<commit_message>
Proposta 3 fecha com as cinco regras integrais
Testando sementes diferentes para a busca da Proposta 3, a semente 7
fecha as oito turmas sem nenhuma exceção — a anterior (20261107) deixava
a 11C1 sem solução dentro do orçamento de nós e obrigava a relaxar nela a
regra 4 (não ceder às vésperas da própria prova).

Com restrições tão apertadas, a semente decide se existe ou não solução
alcançável, e não apenas qual solução sai. Fica fixada em
SEED_PROPOSTA_3, e a skill passa a mandar testar sementes antes de
concluir que uma regra é inviável.

Resultado: zero exceções. Pior caso de cessão 10,7% (contra 23,1% na
Proposta 1); os 8 casos de violação da regra 4 que restavam na 11C1
desapareceram.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Relatorio_Tempos_Cedidos_Proposta_3.xlsx
+++ b/Horario desenvolvido/Relatorio_Tempos_Cedidos_Proposta_3.xlsx
@@ -597,58 +597,58 @@
         <v>95</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.03157894736842105</v>
+        <v>0.04210526315789474</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Artes</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Caro (Carolina Salles Kehl), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Artes</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Caro (Carolina Salles Kehl), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.0625</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="7">
@@ -678,12 +678,12 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Jana (Janaína Souza Silva)</t>
+          <t>JuLa (Júlia Soares Leite Lanzarini de Carvalho)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
@@ -702,12 +702,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>JuLa (Júlia Soares Leite Lanzarini de Carvalho)</t>
+          <t>Jana (Janaína Souza Silva)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
@@ -717,10 +717,10 @@
         <v>32</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.03125</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="10">
@@ -999,10 +999,10 @@
         <v>617</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>0.03079416531604538</v>
+        <v>0.03241491085899514</v>
       </c>
     </row>
   </sheetData>
@@ -1088,82 +1088,82 @@
         <v>95</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.03157894736842105</v>
+        <v>0.04210526315789474</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Caro (Carolina Salles Kehl), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
+          <t>BrSa (Bruno Vianna dos Santos)</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Artes</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>BrSa (Bruno Vianna dos Santos)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>80</v>
+        <v>32</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.0375</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Artes</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Caro (Carolina Salles Kehl), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.0625</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="7">
@@ -1193,49 +1193,49 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
+          <t>JuLa (Júlia Soares Leite Lanzarini de Carvalho)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.04444444444444445</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Apoio</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>JuLa (Júlia Soares Leite Lanzarini de Carvalho)</t>
+          <t>Caro (Carolina Salles Kehl)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.03333333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1246,14 +1246,14 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Caro (Carolina Salles Kehl)</t>
+          <t>FBri (Fábio Luís de Brito)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>0</v>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>FBri (Fábio Luís de Brito)</t>
+          <t>SMo (Samara Costa Moura)</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -1289,19 +1289,19 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Apoio</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>SMo (Samara Costa Moura)</t>
+          <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>0</v>
@@ -1313,19 +1313,19 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Ed.Física</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Ale (Alexandre de Almeida Pereira)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>0</v>
@@ -1337,19 +1337,19 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Ed.Física</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VSi (Vinícius de Paula Silveira)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>0</v>
@@ -1361,19 +1361,19 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>VSi (Vinícius de Paula Silveira)</t>
+          <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>0</v>
@@ -1385,19 +1385,19 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Mar (Marcelo Alonso Morais)</t>
+          <t>APa (Ana Patricia Machado de Pinho Garcia), PaH (Paulo Henrique Sá Júnior), Velo (Rodrigo Veloso)</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="E16" s="6" t="n">
         <v>0</v>
@@ -1409,19 +1409,19 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>APa (Ana Patricia Machado de Pinho Garcia), PaH (Paulo Henrique Sá Júnior), Velo (Rodrigo Veloso)</t>
+          <t>Fab (Fabio Merçon)</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>0</v>
@@ -1433,19 +1433,19 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Fab (Fabio Merçon)</t>
+          <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
@@ -1514,10 +1514,10 @@
         <v>617</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>0.02593192868719611</v>
+        <v>0.02431118314424635</v>
       </c>
     </row>
   </sheetData>
@@ -2810,103 +2810,103 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>Aprof.</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Bea (Beatriz Souza Andrade Maciel)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
         <v>4</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.06451612903225806</v>
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Aprof.</t>
+          <t>DaF</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CBu (Claudia Burkhardt), SGa (Sabrina Gab), Swa (Greta Schwankhaus Oliveira)</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="E4" s="6" t="n">
         <v>3</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.03896103896103896</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>DaF</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), SGa (Sabrina Gab), Swa (Greta Schwankhaus Oliveira)</t>
+          <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>77</v>
+        <v>29</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>3</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.03896103896103896</v>
+        <v>0.103448275862069</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Ver (Verena Alberti)</t>
+          <t>Bea (Beatriz Souza Andrade Maciel)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>3</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.0625</v>
+        <v>0.04838709677419355</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Artes</t>
+          <t>Ed.Física</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -2930,132 +2930,132 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Ale (Alexandre de Almeida Pereira)</t>
+          <t>Cadu (Carlos Eduardo Lima)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
         <v>3</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.0425531914893617</v>
+        <v>0.04166666666666666</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Ed.Física</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ver (Verena Alberti)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.0625</v>
+        <v>0.04166666666666666</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Cadu (Carlos Eduardo Lima)</t>
+          <t>ClaMe (Clarissa Duarte Loureiro de Melo)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
         <v>3</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.04347826086956522</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Mar (Marcelo Alonso Morais)</t>
+          <t>JJ (João Jorge Fernandes Chaves)</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.06896551724137931</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>ClaMe (Clarissa Duarte Loureiro de Melo)</t>
+          <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.04347826086956522</v>
+        <v>0.06451612903225806</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Artes</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>JJ (João Jorge Fernandes Chaves)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
@@ -3065,45 +3065,45 @@
         <v>32</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.0625</v>
+        <v>0.03125</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>AMu (André Barros Mucci)</t>
+          <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.06451612903225806</v>
+        <v>0.02127659574468085</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CAl (Carlos Alberto Linhares da Silva)</t>
+          <t>CBu (Claudia Burkhardt), Swa (Greta Schwankhaus Oliveira), SGa (Sabrina Gab)</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -3122,67 +3122,67 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Proj.Vestibular</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>ACo (Alexandre Braga Badaue Coelho)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>30</v>
+        <v>126</v>
       </c>
       <c r="E16" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>0.03333333333333333</v>
+        <v>0.007936507936507936</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Fil</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
+          <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Fil</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), Swa (Greta Schwankhaus Oliveira), SGa (Sabrina Gab)</t>
+          <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
@@ -3218,19 +3218,19 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Proj.Vestibular</t>
+          <t>Projeto</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>APa (Ana Patricia Machado de Pinho Garcia)</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>126</v>
+        <v>28</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>0</v>
@@ -3242,19 +3242,19 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Projeto</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>APa (Ana Patricia Machado de Pinho Garcia)</t>
+          <t>ACo (Alexandre Braga Badaue Coelho)</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>0</v>
@@ -3299,10 +3299,10 @@
         <v>837</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>0.03703703703703703</v>
+        <v>0.03464755077658303</v>
       </c>
     </row>
   </sheetData>
@@ -3397,73 +3397,73 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Ver (Verena Alberti)</t>
+          <t>PaH (Paulo Henrique Sá Júnior)</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="E4" s="6" t="n">
         <v>3</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.0625</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Artes</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.0625</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>DaF</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Ale (Alexandre de Almeida Pereira)</t>
+          <t>CBu (Claudia Burkhardt), SGa (Sabrina Gab), Swa (Greta Schwankhaus Oliveira)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.04444444444444445</v>
+        <v>0.02597402597402598</v>
       </c>
     </row>
     <row r="7">
@@ -3517,25 +3517,25 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>PaH (Paulo Henrique Sá Júnior)</t>
+          <t>CBu (Claudia Burkhardt), Swa (Greta Schwankhaus Oliveira), SGa (Sabrina Gab)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.03333333333333333</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="10">
@@ -3546,31 +3546,31 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>JJ (João Jorge Fernandes Chaves)</t>
+          <t>ClaMe (Clarissa Duarte Loureiro de Melo)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.0625</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>AMu (André Barros Mucci)</t>
+          <t>JJ (João Jorge Fernandes Chaves)</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -3589,84 +3589,84 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>ACo (Alexandre Braga Badaue Coelho)</t>
+          <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>DaF</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), SGa (Sabrina Gab), Swa (Greta Schwankhaus Oliveira)</t>
+          <t>ACo (Alexandre Braga Badaue Coelho)</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.01298701298701299</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Artes</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), Swa (Greta Schwankhaus Oliveira), SGa (Sabrina Gab)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.03333333333333333</v>
+        <v>0.03125</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CAl (Carlos Alberto Linhares da Silva)</t>
+          <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -3685,43 +3685,43 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Fil</t>
+          <t>Proj.Vestibular</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>16</v>
+        <v>126</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>0</v>
+        <v>0.007936507936507936</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>Fil</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Mar (Marcelo Alonso Morais)</t>
+          <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>0</v>
@@ -3733,19 +3733,19 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Gram</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
+          <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
@@ -3757,19 +3757,19 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Gram</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>ClaMe (Clarissa Duarte Loureiro de Melo)</t>
+          <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>0</v>
@@ -3781,19 +3781,19 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Proj.Vestibular</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ver (Verena Alberti)</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>126</v>
+        <v>48</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>0</v>
@@ -3862,10 +3862,10 @@
         <v>837</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>0.02986857825567503</v>
+        <v>0.03225806451612903</v>
       </c>
     </row>
   </sheetData>
@@ -3936,121 +3936,121 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Proj.Vestibular</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Deb (Debora Borba Linhares)</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>108</v>
+        <v>56</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>4</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.03703703703703703</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>DaF</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Mar (Marcelo Alonso Morais)</t>
+          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="E4" s="6" t="n">
         <v>3</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.07894736842105263</v>
+        <v>0.04411764705882353</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Deb (Debora Borba Linhares)</t>
+          <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>3</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.05357142857142857</v>
+        <v>0.07894736842105263</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Aprof.</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Ale (Alexandre de Almeida Pereira)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.05</v>
+        <v>0.03571428571428571</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>DaF</t>
+          <t>Artes</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.02941176470588235</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="8">
@@ -4080,36 +4080,36 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Wag (Wagner Pinto da Silva)</t>
+          <t>PaH (Paulo Henrique Sá Júnior)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.05263157894736842</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Fab (Fabio Merçon)</t>
+          <t>Bre (Carlos Luiz Silva Brener)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
@@ -4128,60 +4128,60 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Proj.Vestibular</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>AMu (André Barros Mucci)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>28</v>
+        <v>108</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.01851851851851852</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Aprof.</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fab (Fabio Merçon)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Artes</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
@@ -4191,45 +4191,45 @@
         <v>28</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>PaH (Paulo Henrique Sá Júnior)</t>
+          <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
         <v>3</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.02631578947368421</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Bre (Carlos Luiz Silva Brener)</t>
+          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -4296,19 +4296,19 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
+          <t>Wag (Wagner Pinto da Silva)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
@@ -4401,10 +4401,10 @@
         <v>710</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F22" s="11" t="n">
-        <v>0.03661971830985915</v>
+        <v>0.03943661971830986</v>
       </c>
     </row>
   </sheetData>
@@ -4523,7 +4523,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Proj.Vestibular</t>
+          <t>Aprof.</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -4532,37 +4532,37 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>108</v>
+        <v>56</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.03703703703703703</v>
+        <v>0.03571428571428571</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Artes</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Wag (Wagner Pinto da Silva)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>0.07142857142857142</v>
@@ -4571,12 +4571,12 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Mar (Marcelo Alonso Morais)</t>
+          <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
@@ -4595,108 +4595,108 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Isb (Isabela Gomes Bustamante)</t>
+          <t>Cadu (Carlos Eduardo Lima)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Aprof.</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Artes</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Isb (Isabela Gomes Bustamante)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.05263157894736842</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Proj.Vestibular</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Ale (Alexandre de Almeida Pereira)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>40</v>
+        <v>108</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.025</v>
+        <v>0.01851851851851852</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Cadu (Carlos Eduardo Lima)</t>
+          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
@@ -4715,25 +4715,25 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>AMu (André Barros Mucci)</t>
+          <t>Wag (Wagner Pinto da Silva)</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.02380952380952381</v>
       </c>
     </row>
     <row r="14">
@@ -4787,19 +4787,19 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
+          <t>Bre (Carlos Luiz Silva Brener)</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E16" s="6" t="n">
         <v>0</v>
@@ -4816,14 +4816,14 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Bre (Carlos Luiz Silva Brener)</t>
+          <t>JJ (João Jorge Fernandes Chaves)</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>0</v>
@@ -4835,19 +4835,19 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>JJ (João Jorge Fernandes Chaves)</t>
+          <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
@@ -4864,14 +4864,14 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>CAl (Carlos Alberto Linhares da Silva)</t>
+          <t>Fab (Fabio Merçon)</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>0</v>
@@ -4883,12 +4883,12 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Fab (Fabio Merçon)</t>
+          <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">

</xml_diff>

<commit_message>
Regenera Proposta 3 e relatórios com a regra do LP/LIT/RED implementada
Calendário, relatório de trocas de tempo, tabela por turma e relatório
de tempos cedidos, todos regerados com:
- LP/LIT/RED (10C1/10C2, semana <=9, ver regra na skill);
- escalonamento de cessão localizado por turma (não mais global);
- SEED_PROPOSTA_3 = 3;
- correção da contagem em dobro de cessões (Ing/APa na 10C1).

Fecha as 8 turmas. Única exceção, localizada e divulgada no relatório:
10C1 precisou de regra 4 e regra 3 relaxadas, e do teto de cessões
elevado em +1 (só nela — as outras sete turmas cumprem as cinco regras
de cessão integralmente). Verificado com verificar_calendario.py: OK,
sem nenhum PROBLEMA no checklist.
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Relatorio_Tempos_Cedidos_Proposta_3.xlsx
+++ b/Horario desenvolvido/Relatorio_Tempos_Cedidos_Proposta_3.xlsx
@@ -678,12 +678,12 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Jana (Janaína Souza Silva)</t>
+          <t>JuLa (Júlia Soares Leite Lanzarini de Carvalho)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
@@ -702,12 +702,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>JuLa (Júlia Soares Leite Lanzarini de Carvalho)</t>
+          <t>Jana (Janaína Souza Silva)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
@@ -717,34 +717,34 @@
         <v>32</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.03125</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Apoio</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
+          <t>Caro (Carolina Salles Kehl)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.02222222222222222</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -755,14 +755,14 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Caro (Carolina Salles Kehl)</t>
+          <t>FBri (Fábio Luís de Brito)</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>0</v>
@@ -779,7 +779,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>FBri (Fábio Luís de Brito)</t>
+          <t>SMo (Samara Costa Moura)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
@@ -798,19 +798,19 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Apoio</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>SMo (Samara Costa Moura)</t>
+          <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>0</v>
@@ -822,19 +822,19 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Ed.Física</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Ale (Alexandre de Almeida Pereira)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>0</v>
@@ -846,19 +846,19 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Ed.Física</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VSi (Vinícius de Paula Silveira)</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>0</v>
@@ -870,19 +870,19 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>VSi (Vinícius de Paula Silveira)</t>
+          <t>APa (Ana Patricia Machado de Pinho Garcia), PaH (Paulo Henrique Sá Júnior), Velo (Rodrigo Veloso)</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="E16" s="6" t="n">
         <v>0</v>
@@ -894,19 +894,19 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>APa (Ana Patricia Machado de Pinho Garcia), PaH (Paulo Henrique Sá Júnior), Velo (Rodrigo Veloso)</t>
+          <t>Fab (Fabio Merçon)</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>0</v>
@@ -918,19 +918,19 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Fab (Fabio Merçon)</t>
+          <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
@@ -1112,10 +1112,10 @@
         <v>80</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.0375</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="5">
@@ -1514,10 +1514,10 @@
         <v>617</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>0.0226904376012966</v>
+        <v>0.02431118314424635</v>
       </c>
     </row>
   </sheetData>
@@ -1627,10 +1627,10 @@
         <v>54</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.07407407407407407</v>
+        <v>0.1111111111111111</v>
       </c>
     </row>
     <row r="5">
@@ -1651,82 +1651,82 @@
         <v>28</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.1071428571428571</v>
+        <v>0.1428571428571428</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Ed.Física</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VSi (Vinícius de Paula Silveira)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.1153846153846154</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Ed.Física</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>VSi (Vinícius de Paula Silveira)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>BrSa (Bruno Vianna dos Santos)</t>
+          <t>Mlo (Marcelo Rios Lopes)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="9">
@@ -1804,12 +1804,12 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Mlo (Marcelo Rios Lopes)</t>
+          <t>ALu (Ana Lúcia Fonseca de Castro)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
@@ -1828,25 +1828,25 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ALu (Ana Lúcia Fonseca de Castro)</t>
+          <t>BrSa (Bruno Vianna dos Santos)</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.02380952380952381</v>
       </c>
     </row>
     <row r="14">
@@ -2125,10 +2125,10 @@
         <v>598</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>0.04682274247491638</v>
+        <v>0.05351170568561873</v>
       </c>
     </row>
   </sheetData>
@@ -2415,36 +2415,36 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Lza (Luiza Maria Abreu de Mattos)</t>
+          <t>Mlo (Marcelo Rios Lopes)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.025</v>
+        <v>0.03571428571428571</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Mlo (Marcelo Rios Lopes)</t>
+          <t>ALu (Ana Lúcia Fonseca de Castro)</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
@@ -2463,43 +2463,43 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Apoio</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>ALu (Ana Lúcia Fonseca de Castro)</t>
+          <t>SGa (Sabrina Gab)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.03571428571428571</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Apoio</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>SGa (Sabrina Gab)</t>
+          <t>Lza (Luiza Maria Abreu de Mattos)</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>0</v>
@@ -2736,10 +2736,10 @@
         <v>598</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>0.04347826086956522</v>
+        <v>0.04180602006688963</v>
       </c>
     </row>
   </sheetData>
@@ -2825,58 +2825,58 @@
         <v>63</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.07936507936507936</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>DaF</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), SGa (Sabrina Gab), Swa (Greta Schwankhaus Oliveira)</t>
+          <t>Bea (Beatriz Souza Andrade Maciel)</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.03896103896103896</v>
+        <v>0.06451612903225806</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>DaF</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Mar (Marcelo Alonso Morais)</t>
+          <t>CBu (Claudia Burkhardt), SGa (Sabrina Gab), Swa (Greta Schwankhaus Oliveira)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>3</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.103448275862069</v>
+        <v>0.03896103896103896</v>
       </c>
     </row>
     <row r="6">
@@ -2906,31 +2906,31 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Bea (Beatriz Souza Andrade Maciel)</t>
+          <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.04838709677419355</v>
+        <v>0.0425531914893617</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Artes</t>
+          <t>Ed.Física</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -2954,49 +2954,49 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Ed.Física</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Cadu (Carlos Eduardo Lima)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.0625</v>
+        <v>0.04166666666666666</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Cadu (Carlos Eduardo Lima)</t>
+          <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.06896551724137931</v>
       </c>
     </row>
     <row r="11">
@@ -3026,108 +3026,108 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>JJ (João Jorge Fernandes Chaves)</t>
+          <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.0625</v>
+        <v>0.06451612903225806</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>AMu (André Barros Mucci)</t>
+          <t>ACo (Alexandre Braga Badaue Coelho)</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.06451612903225806</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Ale (Alexandre de Almeida Pereira)</t>
+          <t>JJ (João Jorge Fernandes Chaves)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.02127659574468085</v>
+        <v>0.03125</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Proj.Vestibular</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), Swa (Greta Schwankhaus Oliveira), SGa (Sabrina Gab)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>30</v>
+        <v>126</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.03333333333333333</v>
+        <v>0.007936507936507936</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>ACo (Alexandre Braga Badaue Coelho)</t>
+          <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
@@ -3146,19 +3146,19 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Fil</t>
+          <t>Artes</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>0</v>
@@ -3170,19 +3170,19 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Gram</t>
+          <t>Fil</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
+          <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
@@ -3194,19 +3194,19 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Proj.Vestibular</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CBu (Claudia Burkhardt), Swa (Greta Schwankhaus Oliveira), SGa (Sabrina Gab)</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>126</v>
+        <v>30</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>0</v>
@@ -3218,19 +3218,19 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Projeto</t>
+          <t>Gram</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>APa (Ana Patricia Machado de Pinho Garcia)</t>
+          <t>Raf (Rafael Alverne Freitas de Albuquerque)</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>0</v>
@@ -3242,19 +3242,19 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Projeto</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>CAl (Carlos Alberto Linhares da Silva)</t>
+          <t>APa (Ana Patricia Machado de Pinho Garcia)</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>0</v>
@@ -3299,10 +3299,10 @@
         <v>837</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>0.03584229390681003</v>
+        <v>0.03823178016726404</v>
       </c>
     </row>
   </sheetData>
@@ -3388,322 +3388,322 @@
         <v>63</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.07936507936507936</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>PaH (Paulo Henrique Sá Júnior)</t>
+          <t>Ver (Verena Alberti)</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="E4" s="6" t="n">
         <v>3</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.05</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Artes</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.0625</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Ed.Física</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Ale (Alexandre de Almeida Pereira)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.04444444444444445</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>DaF</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), SGa (Sabrina Gab), Swa (Greta Schwankhaus Oliveira)</t>
+          <t>Cadu (Carlos Eduardo Lima)</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.02597402597402598</v>
+        <v>0.04166666666666666</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Ed.Física</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ClaMe (Clarissa Duarte Loureiro de Melo)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.0625</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Cadu (Carlos Eduardo Lima)</t>
+          <t>JJ (João Jorge Fernandes Chaves)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), Swa (Greta Schwankhaus Oliveira), SGa (Sabrina Gab)</t>
+          <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Ver (Verena Alberti)</t>
+          <t>ACo (Alexandre Braga Badaue Coelho)</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>DaF</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>JJ (João Jorge Fernandes Chaves)</t>
+          <t>CBu (Claudia Burkhardt), SGa (Sabrina Gab), Swa (Greta Schwankhaus Oliveira)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>32</v>
+        <v>77</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.0625</v>
+        <v>0.01298701298701299</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ClaMe (Clarissa Duarte Loureiro de Melo)</t>
+          <t>CBu (Claudia Burkhardt), Swa (Greta Schwankhaus Oliveira), SGa (Sabrina Gab)</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.02222222222222222</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>AMu (André Barros Mucci)</t>
+          <t>PaH (Paulo Henrique Sá Júnior)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.03125</v>
+        <v>0.01666666666666667</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Proj.Vestibular</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CAl (Carlos Alberto Linhares da Silva)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>32</v>
+        <v>126</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.03125</v>
+        <v>0.007936507936507936</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Artes</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>ACo (Alexandre Braga Badaue Coelho)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>0.03333333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -3781,19 +3781,19 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Proj.Vestibular</t>
+          <t>Projeto</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>APa (Ana Patricia Machado de Pinho Garcia)</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>126</v>
+        <v>28</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>0</v>
@@ -3805,19 +3805,19 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Projeto</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>APa (Ana Patricia Machado de Pinho Garcia)</t>
+          <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>0</v>
@@ -3936,132 +3936,132 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Proj.Vestibular</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Deb (Debora Borba Linhares)</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>108</v>
+        <v>56</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>5</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.04629629629629629</v>
+        <v>0.08928571428571429</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>Aprof.</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Mar (Marcelo Alonso Morais)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="E4" s="6" t="n">
         <v>3</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.07894736842105263</v>
+        <v>0.05357142857142857</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>DaF</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Ale (Alexandre de Almeida Pereira)</t>
+          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>2</v>
-      </c>
       <c r="F5" s="5" t="n">
-        <v>0.05</v>
+        <v>0.04411764705882353</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>DaF</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
+          <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.02941176470588235</v>
+        <v>0.07894736842105263</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Cadu (Carlos Eduardo Lima)</t>
+          <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>AMu (André Barros Mucci)</t>
+          <t>Cadu (Carlos Eduardo Lima)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
@@ -4080,36 +4080,36 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Aprof.</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Bre (Carlos Luiz Silva Brener)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Artes</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fab (Fabio Merçon)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
@@ -4119,130 +4119,130 @@
         <v>28</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Wag (Wagner Pinto da Silva)</t>
+          <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.02380952380952381</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>Artes</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>PaH (Paulo Henrique Sá Júnior)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.02631578947368421</v>
+        <v>0.03571428571428571</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Bre (Carlos Luiz Silva Brener)</t>
+          <t>Wag (Wagner Pinto da Silva)</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.02380952380952381</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Deb (Debora Borba Linhares)</t>
+          <t>PaH (Paulo Henrique Sá Júnior)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.02631578947368421</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Proj.Vestibular</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Fab (Fabio Merçon)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>28</v>
+        <v>108</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.009259259259259259</v>
       </c>
     </row>
     <row r="16">
@@ -4401,10 +4401,10 @@
         <v>710</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F22" s="11" t="n">
-        <v>0.0323943661971831</v>
+        <v>0.03943661971830986</v>
       </c>
     </row>
   </sheetData>
@@ -4499,49 +4499,49 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Proj.Vestibular</t>
+          <t>DaF</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>108</v>
+        <v>68</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.05555555555555555</v>
+        <v>0.07352941176470588</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>DaF</t>
+          <t>Aprof.</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>3</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.04411764705882353</v>
+        <v>0.05357142857142857</v>
       </c>
     </row>
     <row r="6">
@@ -4571,103 +4571,103 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Ale (Alexandre de Almeida Pereira)</t>
+          <t>Cadu (Carlos Eduardo Lima)</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.05</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Cadu (Carlos Eduardo Lima)</t>
+          <t>Mar (Marcelo Alonso Morais)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Mar (Marcelo Alonso Morais)</t>
+          <t>Isb (Isabela Gomes Bustamante)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.05</v>
+        <v>0.05263157894736842</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>Artes</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Isb (Isabela Gomes Bustamante)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.03571428571428571</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Aprof.</t>
+          <t>Proj.Vestibular</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -4676,27 +4676,27 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>56</v>
+        <v>108</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.009259259259259259</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Artes</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>AMu (André Barros Mucci)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
@@ -4715,36 +4715,36 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Fab (Fabio Merçon)</t>
+          <t>Ale (Alexandre de Almeida Pereira)</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.03571428571428571</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Ed.Física</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>AMu (André Barros Mucci)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
@@ -4754,28 +4754,28 @@
         <v>28</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.03571428571428571</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Ed.Física</t>
+          <t>Fil</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>0</v>
@@ -4787,19 +4787,19 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Fil</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>LAn (Luiz Antônio Andrade de Oliveira)</t>
+          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="E16" s="6" t="n">
         <v>0</v>
@@ -4811,19 +4811,19 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>CBu (Claudia Burkhardt), EFr (Wera Elisabeth Catharina Fricke Bispo Oliveira), Eth (Ethel Vera Figur Driesen)</t>
+          <t>Bre (Carlos Luiz Silva Brener)</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>0</v>
@@ -4840,14 +4840,14 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Bre (Carlos Luiz Silva Brener)</t>
+          <t>JJ (João Jorge Fernandes Chaves)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
@@ -4859,19 +4859,19 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>JJ (João Jorge Fernandes Chaves)</t>
+          <t>CAl (Carlos Alberto Linhares da Silva)</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>0</v>
@@ -4888,14 +4888,14 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>CAl (Carlos Alberto Linhares da Silva)</t>
+          <t>Fab (Fabio Merçon)</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>0</v>
@@ -4940,10 +4940,10 @@
         <v>710</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F22" s="11" t="n">
-        <v>0.04225352112676056</v>
+        <v>0.03661971830985915</v>
       </c>
     </row>
   </sheetData>

</xml_diff>